<commit_message>
Refresh example reports from current template
</commit_message>
<xml_diff>
--- a/examples/qualibact_ecoli/real_panel/report/report.xlsx
+++ b/examples/qualibact_ecoli/real_panel/report/report.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="D2" t="b">
@@ -590,12 +590,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>no_of_contigs &gt;600.0; Total_Coding_Sequences &gt;5800.0</t>
+          <t>Checkm.GC</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -669,12 +669,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>no_of_contigs &gt;670.0; Total_Coding_Sequences &gt;5800.0; Genome_Size &gt;5700000.0</t>
+          <t>none</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="D4" t="b">
@@ -748,12 +748,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Checkm.GC</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="D2" t="b">
@@ -938,12 +938,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>no_of_contigs &gt;600.0; Total_Coding_Sequences &gt;5800.0</t>
+          <t>Checkm.GC</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1017,12 +1017,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>no_of_contigs &gt;670.0; Total_Coding_Sequences &gt;5800.0; Genome_Size &gt;5700000.0</t>
+          <t>none</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="D4" t="b">
@@ -1096,12 +1096,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Checkm.GC</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CH4"/>
+  <dimension ref="A1:CQ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1157,395 +1157,440 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>Checkm.Total_Coding_Sequences.check</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Quast.# contigs (&gt;= 0 bp).check</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Quast.GC (%).check</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Quast.N50.check</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Quast.Ns per 100 kbp.check</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Quast.Total length (&gt;= 0 bp).check</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Speciator.confidence.check</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Speciator.genusName.check</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Speciator.speciesName.check</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Sylph.number_of_genomes.check</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Sylph.sequence_abundances.check</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Sylph.species_name.check</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Checkm.# contigs</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Checkm.Completeness</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Checkm.Contamination</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Checkm.Contig_N50</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Checkm.GC</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Checkm.GC_Content</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Checkm.Genome size (bp)</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Checkm.Genome_Size</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Checkm.N50 (scaffolds)</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Checkm.Total_Coding_Sequences</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Checkm.Total_Contigs</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Checkm.all_checks_passed</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Depth.Depth</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Depth.Read_type</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Depth.all_checks_passed</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Quast.# contigs</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Quast.# contigs (&gt;= 0 bp)</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Quast.GC (%)</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Quast.Largest contig</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Quast.N50</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Quast.Total length</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Quast.Total length (&gt;= 0 bp)</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Quast.all_checks_passed</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>Speciator.all_checks_passed</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>Speciator.confidence</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Speciator.speciesName</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Sylph.all_checks_passed</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Sylph.genomes</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Sylph.number_of_genomes</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>Sylph.species_name</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>Sylph.taxonomic_abundances</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>Sylph.top_adjusted_ani</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>Sylph.top_species</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>Sylph.top_taxonomic_abundance</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>all_checks_passed</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>qualibact_N50</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>qualibact_completeness_specific</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>qualibact_contamination</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>qualibact_contigs</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>qualibact_gc_content</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>qualibact_genome_size</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>qualibact_reasons</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>qualibact_species_sylph</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>qualibact_tier</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>speccheck_assembly_type</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>speccheck_baseline_checks_passed</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>speccheck_baseline_overridden_count</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
         <is>
           <t>speccheck_criteria_file</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>speccheck_criteria_sha256</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>speccheck_fail_on_not_evaluated</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>speccheck_failure_count</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>speccheck_failure_reasons</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
         <is>
           <t>speccheck_input_file_count</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>speccheck_not_evaluated_count</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>speccheck_overall_status</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
         <is>
           <t>speccheck_species_checks_available</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>speccheck_species_checks_passed</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>speccheck_threshold_fallback_used</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>speccheck_threshold_scheme</t>
         </is>
       </c>
-      <c r="BV1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>speccheck_threshold_source</t>
         </is>
       </c>
-      <c r="BW1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>speccheck_version</t>
         </is>
       </c>
-      <c r="BX1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>speccheck_warning_count</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr">
+        <is>
+          <t>speccheck_warning_reasons</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr">
         <is>
           <t>qualibact_compat_tier</t>
         </is>
       </c>
-      <c r="BY1" t="inlineStr">
+      <c r="CF1" t="inlineStr">
         <is>
           <t>qualibact_compat_passed</t>
         </is>
       </c>
-      <c r="BZ1" t="inlineStr">
+      <c r="CG1" t="inlineStr">
         <is>
           <t>qualibact_compat_reasons</t>
         </is>
       </c>
-      <c r="CA1" t="inlineStr">
+      <c r="CH1" t="inlineStr">
         <is>
           <t>qualibact_compat_warn_policy</t>
         </is>
       </c>
-      <c r="CB1" t="inlineStr">
+      <c r="CI1" t="inlineStr">
         <is>
           <t>qualibact_compat_source</t>
         </is>
       </c>
-      <c r="CC1" t="inlineStr">
+      <c r="CJ1" t="inlineStr">
+        <is>
+          <t>qualibact_compat_metrics_evaluated</t>
+        </is>
+      </c>
+      <c r="CK1" t="inlineStr">
+        <is>
+          <t>qualibact_compat_metrics_missing</t>
+        </is>
+      </c>
+      <c r="CL1" t="inlineStr">
         <is>
           <t>overall_qc</t>
         </is>
       </c>
-      <c r="CD1" t="inlineStr">
+      <c r="CM1" t="inlineStr">
         <is>
           <t>baseline_qc</t>
         </is>
       </c>
-      <c r="CE1" t="inlineStr">
+      <c r="CN1" t="inlineStr">
         <is>
           <t>species</t>
         </is>
       </c>
-      <c r="CF1" t="inlineStr">
+      <c r="CO1" t="inlineStr">
         <is>
           <t>species_confidence</t>
         </is>
       </c>
-      <c r="CG1" t="inlineStr">
+      <c r="CP1" t="inlineStr">
         <is>
           <t>threshold_source</t>
         </is>
       </c>
-      <c r="CH1" t="inlineStr">
+      <c r="CQ1" t="inlineStr">
         <is>
           <t>reason_summary</t>
         </is>
@@ -1574,7 +1619,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1642,82 +1687,82 @@
           <t>PASSED</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
         <v>304</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>100</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>0.33</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>112461</v>
-      </c>
-      <c r="W2" t="n">
-        <v>50</v>
       </c>
       <c r="X2" t="n">
         <v>50</v>
       </c>
       <c r="Y2" t="n">
-        <v>5575799</v>
+        <v>50</v>
       </c>
       <c r="Z2" t="n">
         <v>5575799</v>
       </c>
       <c r="AA2" t="n">
+        <v>5575799</v>
+      </c>
+      <c r="AB2" t="n">
         <v>112461</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>5677</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>304</v>
       </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AE2" t="n">
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
         <v>48.91</v>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AH2" t="n">
-        <v>304</v>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
       </c>
       <c r="AI2" t="n">
         <v>304</v>
       </c>
       <c r="AJ2" t="n">
+        <v>304</v>
+      </c>
+      <c r="AK2" t="n">
         <v>50.38</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AL2" t="n">
         <v>288131</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AM2" t="n">
         <v>112461</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>5575799</v>
       </c>
       <c r="AN2" t="n">
         <v>5575799</v>
       </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
+      <c r="AO2" t="n">
+        <v>5575799</v>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
@@ -1726,186 +1771,221 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
           <t>good</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
       <c r="AT2" t="inlineStr">
         <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
           <t>GCF_003697165.2</t>
         </is>
       </c>
-      <c r="AU2" t="n">
+      <c r="AV2" t="n">
         <v>1</v>
       </c>
-      <c r="AV2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AW2" t="n">
+      <c r="AX2" t="n">
         <v>100</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="AY2" t="n">
         <v>97.41</v>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AZ2" t="n">
+      <c r="BA2" t="n">
         <v>100</v>
       </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="BB2" t="n">
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="BC2" t="n">
         <v>114262</v>
       </c>
-      <c r="BC2" t="n">
+      <c r="BD2" t="n">
         <v>100</v>
       </c>
-      <c r="BD2" t="n">
+      <c r="BE2" t="n">
         <v>0.31</v>
       </c>
-      <c r="BE2" t="n">
+      <c r="BF2" t="n">
         <v>665</v>
       </c>
-      <c r="BF2" t="n">
+      <c r="BG2" t="n">
         <v>50.4387</v>
       </c>
-      <c r="BG2" t="n">
+      <c r="BH2" t="n">
         <v>5695351</v>
       </c>
-      <c r="BH2" t="inlineStr">
+      <c r="BI2" t="inlineStr">
         <is>
           <t>no_of_contigs &gt;600.0; Total_Coding_Sequences &gt;5800.0</t>
         </is>
       </c>
-      <c r="BI2" t="inlineStr">
+      <c r="BJ2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="BJ2" t="inlineStr">
+      <c r="BK2" t="inlineStr">
         <is>
           <t>WARN</t>
         </is>
       </c>
-      <c r="BK2" t="inlineStr">
+      <c r="BL2" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="BL2" t="b">
+      <c r="BM2" t="b">
         <v>1</v>
       </c>
-      <c r="BM2" t="inlineStr">
+      <c r="BN2" t="n">
+        <v>9</v>
+      </c>
+      <c r="BO2" t="inlineStr">
         <is>
           <t>/gpfs3/well/aanensen/users/rva470/speccheck/speccheck/config/criteria.csv</t>
         </is>
       </c>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>94ca578103ce4fcd06e80c89e7d76ef7f29a6df0799aacfa92c0acd625506607</t>
-        </is>
-      </c>
-      <c r="BO2" t="b">
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>6b21d56411908a87ca67636a2ee6c7712040ce5da009204f4dd3fc0762b64b0e</t>
+        </is>
+      </c>
+      <c r="BQ2" t="b">
         <v>0</v>
       </c>
-      <c r="BP2" t="n">
+      <c r="BR2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>Checkm.GC &gt;=50.09 (qualibact-v1.0)</t>
+        </is>
+      </c>
+      <c r="BT2" t="n">
         <v>5</v>
       </c>
-      <c r="BQ2" t="n">
+      <c r="BU2" t="n">
         <v>0</v>
       </c>
-      <c r="BR2" t="b">
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="BW2" t="b">
         <v>1</v>
       </c>
-      <c r="BS2" t="b">
+      <c r="BX2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY2" t="b">
         <v>1</v>
       </c>
-      <c r="BT2" t="b">
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="CC2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>Checkm.GC &gt;=50.25 (qualibact-v1.0)</t>
+        </is>
+      </c>
+      <c r="CE2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="CF2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="CG2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="CH2" t="inlineStr">
+        <is>
+          <t>warn-as-warn</t>
+        </is>
+      </c>
+      <c r="CI2" t="inlineStr">
+        <is>
+          <t>Pinned QualiBact scheme for Escherichia coli</t>
+        </is>
+      </c>
+      <c r="CJ2" t="n">
+        <v>8</v>
+      </c>
+      <c r="CK2" t="n">
         <v>0</v>
       </c>
-      <c r="BU2" t="inlineStr">
-        <is>
-          <t>qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>1.2.5</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr">
+      <c r="CL2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="BY2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr">
-        <is>
-          <t>warn-as-warn</t>
-        </is>
-      </c>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia_coli qualibact-v1.0 ATB tier logic</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="CD2" t="b">
+      <c r="CM2" t="b">
         <v>1</v>
       </c>
-      <c r="CE2" t="inlineStr">
+      <c r="CN2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="CF2" t="inlineStr">
+      <c r="CO2" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="CG2" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="CH2" t="inlineStr">
-        <is>
-          <t>no_of_contigs &gt;600.0; Total_Coding_Sequences &gt;5800.0</t>
+      <c r="CP2" t="inlineStr">
+        <is>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CQ2" t="inlineStr">
+        <is>
+          <t>Checkm.GC</t>
         </is>
       </c>
     </row>
@@ -2000,82 +2080,82 @@
           <t>PASSED</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
         <v>302</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>100</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>0.38</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>126621</v>
-      </c>
-      <c r="W3" t="n">
-        <v>51</v>
       </c>
       <c r="X3" t="n">
         <v>51</v>
       </c>
       <c r="Y3" t="n">
-        <v>5625334</v>
+        <v>51</v>
       </c>
       <c r="Z3" t="n">
         <v>5625334</v>
       </c>
       <c r="AA3" t="n">
+        <v>5625334</v>
+      </c>
+      <c r="AB3" t="n">
         <v>126621</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>5715</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>302</v>
       </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AE3" t="n">
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AF3" t="n">
         <v>67.09999999999999</v>
       </c>
-      <c r="AF3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AH3" t="n">
-        <v>302</v>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
       </c>
       <c r="AI3" t="n">
         <v>302</v>
       </c>
       <c r="AJ3" t="n">
+        <v>302</v>
+      </c>
+      <c r="AK3" t="n">
         <v>50.51</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AL3" t="n">
         <v>312337</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="AM3" t="n">
         <v>126621</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>5625334</v>
       </c>
       <c r="AN3" t="n">
         <v>5625334</v>
       </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
+      <c r="AO3" t="n">
+        <v>5625334</v>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
@@ -2084,186 +2164,221 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
           <t>good</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr">
+      <c r="AS3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AS3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
       <c r="AT3" t="inlineStr">
         <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
           <t>GCF_003697165.2</t>
         </is>
       </c>
-      <c r="AU3" t="n">
+      <c r="AV3" t="n">
         <v>1</v>
       </c>
-      <c r="AV3" t="inlineStr">
+      <c r="AW3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AW3" t="n">
+      <c r="AX3" t="n">
         <v>100</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="AY3" t="n">
         <v>97.38</v>
       </c>
-      <c r="AY3" t="inlineStr">
+      <c r="AZ3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AZ3" t="n">
+      <c r="BA3" t="n">
         <v>100</v>
       </c>
-      <c r="BA3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="BB3" t="n">
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="BC3" t="n">
         <v>126621</v>
       </c>
-      <c r="BC3" t="n">
+      <c r="BD3" t="n">
         <v>100</v>
       </c>
-      <c r="BD3" t="n">
+      <c r="BE3" t="n">
         <v>0.4</v>
       </c>
-      <c r="BE3" t="n">
+      <c r="BF3" t="n">
         <v>679</v>
       </c>
-      <c r="BF3" t="n">
+      <c r="BG3" t="n">
         <v>50.5585</v>
       </c>
-      <c r="BG3" t="n">
+      <c r="BH3" t="n">
         <v>5738641</v>
       </c>
-      <c r="BH3" t="inlineStr">
+      <c r="BI3" t="inlineStr">
         <is>
           <t>no_of_contigs &gt;670.0; Total_Coding_Sequences &gt;5800.0; Genome_Size &gt;5700000.0</t>
         </is>
       </c>
-      <c r="BI3" t="inlineStr">
+      <c r="BJ3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="BJ3" t="inlineStr">
+      <c r="BK3" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="BK3" t="inlineStr">
+      <c r="BL3" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="BL3" t="b">
+      <c r="BM3" t="b">
         <v>1</v>
       </c>
-      <c r="BM3" t="inlineStr">
+      <c r="BN3" t="n">
+        <v>9</v>
+      </c>
+      <c r="BO3" t="inlineStr">
         <is>
           <t>/gpfs3/well/aanensen/users/rva470/speccheck/speccheck/config/criteria.csv</t>
         </is>
       </c>
-      <c r="BN3" t="inlineStr">
-        <is>
-          <t>94ca578103ce4fcd06e80c89e7d76ef7f29a6df0799aacfa92c0acd625506607</t>
-        </is>
-      </c>
-      <c r="BO3" t="b">
+      <c r="BP3" t="inlineStr">
+        <is>
+          <t>6b21d56411908a87ca67636a2ee6c7712040ce5da009204f4dd3fc0762b64b0e</t>
+        </is>
+      </c>
+      <c r="BQ3" t="b">
         <v>0</v>
       </c>
-      <c r="BP3" t="n">
+      <c r="BR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="BT3" t="n">
         <v>5</v>
       </c>
-      <c r="BQ3" t="n">
+      <c r="BU3" t="n">
         <v>0</v>
       </c>
-      <c r="BR3" t="b">
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="BW3" t="b">
         <v>1</v>
       </c>
-      <c r="BS3" t="b">
+      <c r="BX3" t="b">
         <v>1</v>
       </c>
-      <c r="BT3" t="b">
+      <c r="BY3" t="b">
+        <v>1</v>
+      </c>
+      <c r="BZ3" t="inlineStr">
+        <is>
+          <t>qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr">
+        <is>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CB3" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="CC3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD3" t="inlineStr">
+        <is>
+          <t>Checkm.GC &lt;=50.88 (qualibact-v1.0)</t>
+        </is>
+      </c>
+      <c r="CE3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="CF3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="CG3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="CH3" t="inlineStr">
+        <is>
+          <t>warn-as-warn</t>
+        </is>
+      </c>
+      <c r="CI3" t="inlineStr">
+        <is>
+          <t>Pinned QualiBact scheme for Escherichia coli</t>
+        </is>
+      </c>
+      <c r="CJ3" t="n">
+        <v>8</v>
+      </c>
+      <c r="CK3" t="n">
         <v>0</v>
       </c>
-      <c r="BU3" t="inlineStr">
-        <is>
-          <t>qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="BV3" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="BW3" t="inlineStr">
-        <is>
-          <t>1.2.5</t>
-        </is>
-      </c>
-      <c r="BX3" t="inlineStr">
+      <c r="CL3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="BY3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="BZ3" t="inlineStr">
+      <c r="CM3" t="b">
+        <v>1</v>
+      </c>
+      <c r="CN3" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="CO3" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="CP3" t="inlineStr">
+        <is>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CQ3" t="inlineStr">
         <is>
           <t>none</t>
-        </is>
-      </c>
-      <c r="CA3" t="inlineStr">
-        <is>
-          <t>warn-as-warn</t>
-        </is>
-      </c>
-      <c r="CB3" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia_coli qualibact-v1.0 ATB tier logic</t>
-        </is>
-      </c>
-      <c r="CC3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="CD3" t="b">
-        <v>1</v>
-      </c>
-      <c r="CE3" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="CF3" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="CG3" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="CH3" t="inlineStr">
-        <is>
-          <t>no_of_contigs &gt;670.0; Total_Coding_Sequences &gt;5800.0; Genome_Size &gt;5700000.0</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2405,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2358,82 +2473,82 @@
           <t>PASSED</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
         <v>121</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>100</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>0.21</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>119508</v>
-      </c>
-      <c r="W4" t="n">
-        <v>50</v>
       </c>
       <c r="X4" t="n">
         <v>50</v>
       </c>
       <c r="Y4" t="n">
-        <v>5023793</v>
+        <v>50</v>
       </c>
       <c r="Z4" t="n">
         <v>5023793</v>
       </c>
       <c r="AA4" t="n">
+        <v>5023793</v>
+      </c>
+      <c r="AB4" t="n">
         <v>119508</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>4800</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>121</v>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AE4" t="n">
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="AF4" t="n">
         <v>47.74</v>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AH4" t="n">
-        <v>121</v>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
       </c>
       <c r="AI4" t="n">
         <v>121</v>
       </c>
       <c r="AJ4" t="n">
+        <v>121</v>
+      </c>
+      <c r="AK4" t="n">
         <v>50.41</v>
       </c>
-      <c r="AK4" t="n">
+      <c r="AL4" t="n">
         <v>684542</v>
       </c>
-      <c r="AL4" t="n">
+      <c r="AM4" t="n">
         <v>119508</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>5023793</v>
       </c>
       <c r="AN4" t="n">
         <v>5023793</v>
       </c>
-      <c r="AO4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
+      <c r="AO4" t="n">
+        <v>5023793</v>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
@@ -2442,186 +2557,221 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
           <t>good</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr">
+      <c r="AS4" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AS4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
       <c r="AT4" t="inlineStr">
         <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
           <t>GCF_003697165.2</t>
         </is>
       </c>
-      <c r="AU4" t="n">
+      <c r="AV4" t="n">
         <v>1</v>
       </c>
-      <c r="AV4" t="inlineStr">
+      <c r="AW4" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AW4" t="n">
+      <c r="AX4" t="n">
         <v>100</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="AY4" t="n">
         <v>97.25</v>
       </c>
-      <c r="AY4" t="inlineStr">
+      <c r="AZ4" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="AZ4" t="n">
+      <c r="BA4" t="n">
         <v>100</v>
       </c>
-      <c r="BA4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="BB4" t="n">
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="BC4" t="n">
         <v>120461</v>
       </c>
-      <c r="BC4" t="n">
+      <c r="BD4" t="n">
         <v>100</v>
       </c>
-      <c r="BD4" t="n">
+      <c r="BE4" t="n">
         <v>0.21</v>
       </c>
-      <c r="BE4" t="n">
+      <c r="BF4" t="n">
         <v>184</v>
       </c>
-      <c r="BF4" t="n">
+      <c r="BG4" t="n">
         <v>50.4198</v>
       </c>
-      <c r="BG4" t="n">
+      <c r="BH4" t="n">
         <v>5043262</v>
       </c>
-      <c r="BH4" t="inlineStr">
+      <c r="BI4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="BI4" t="inlineStr">
+      <c r="BJ4" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="BJ4" t="inlineStr">
+      <c r="BK4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="BK4" t="inlineStr">
+      <c r="BL4" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="BL4" t="b">
+      <c r="BM4" t="b">
         <v>1</v>
       </c>
-      <c r="BM4" t="inlineStr">
+      <c r="BN4" t="n">
+        <v>9</v>
+      </c>
+      <c r="BO4" t="inlineStr">
         <is>
           <t>/gpfs3/well/aanensen/users/rva470/speccheck/speccheck/config/criteria.csv</t>
         </is>
       </c>
-      <c r="BN4" t="inlineStr">
-        <is>
-          <t>94ca578103ce4fcd06e80c89e7d76ef7f29a6df0799aacfa92c0acd625506607</t>
-        </is>
-      </c>
-      <c r="BO4" t="b">
+      <c r="BP4" t="inlineStr">
+        <is>
+          <t>6b21d56411908a87ca67636a2ee6c7712040ce5da009204f4dd3fc0762b64b0e</t>
+        </is>
+      </c>
+      <c r="BQ4" t="b">
         <v>0</v>
       </c>
-      <c r="BP4" t="n">
+      <c r="BR4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS4" t="inlineStr">
+        <is>
+          <t>Checkm.GC &gt;=50.09 (qualibact-v1.0)</t>
+        </is>
+      </c>
+      <c r="BT4" t="n">
         <v>5</v>
       </c>
-      <c r="BQ4" t="n">
+      <c r="BU4" t="n">
         <v>0</v>
       </c>
-      <c r="BR4" t="b">
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="BW4" t="b">
         <v>1</v>
       </c>
-      <c r="BS4" t="b">
+      <c r="BX4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY4" t="b">
         <v>1</v>
       </c>
-      <c r="BT4" t="b">
+      <c r="BZ4" t="inlineStr">
+        <is>
+          <t>qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CA4" t="inlineStr">
+        <is>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CB4" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="CC4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD4" t="inlineStr">
+        <is>
+          <t>Checkm.GC &gt;=50.25 (qualibact-v1.0)</t>
+        </is>
+      </c>
+      <c r="CE4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="CF4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="CG4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="CH4" t="inlineStr">
+        <is>
+          <t>warn-as-warn</t>
+        </is>
+      </c>
+      <c r="CI4" t="inlineStr">
+        <is>
+          <t>Pinned QualiBact scheme for Escherichia coli</t>
+        </is>
+      </c>
+      <c r="CJ4" t="n">
+        <v>8</v>
+      </c>
+      <c r="CK4" t="n">
         <v>0</v>
       </c>
-      <c r="BU4" t="inlineStr">
-        <is>
-          <t>qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="BV4" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="BW4" t="inlineStr">
-        <is>
-          <t>1.2.5</t>
-        </is>
-      </c>
-      <c r="BX4" t="inlineStr">
+      <c r="CL4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="BY4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="BZ4" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="CA4" t="inlineStr">
-        <is>
-          <t>warn-as-warn</t>
-        </is>
-      </c>
-      <c r="CB4" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia_coli qualibact-v1.0 ATB tier logic</t>
-        </is>
-      </c>
-      <c r="CC4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="CD4" t="b">
+      <c r="CM4" t="b">
         <v>1</v>
       </c>
-      <c r="CE4" t="inlineStr">
+      <c r="CN4" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="CF4" t="inlineStr">
+      <c r="CO4" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="CG4" t="inlineStr">
-        <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
-        </is>
-      </c>
-      <c r="CH4" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="CP4" t="inlineStr">
+        <is>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
+        </is>
+      </c>
+      <c r="CQ4" t="inlineStr">
+        <is>
+          <t>Checkm.GC</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2839,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2714,12 +2864,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2923,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2798,12 +2948,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
     </row>

</xml_diff>